<commit_message>
Fix Department acronym casing (IT/HR) after str.title()
</commit_message>
<xml_diff>
--- a/financial_report.xlsx
+++ b/financial_report.xlsx
@@ -886,7 +886,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3311,7 +3311,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -4173,7 +4173,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -4837,7 +4837,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -4969,7 +4969,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -5002,7 +5002,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -5662,7 +5662,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -5794,7 +5794,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -5827,7 +5827,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -5860,7 +5860,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -6058,7 +6058,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -6817,7 +6817,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -6949,7 +6949,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -7217,7 +7217,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -7481,7 +7481,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -7580,7 +7580,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -7613,7 +7613,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
@@ -8207,7 +8207,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -8273,7 +8273,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -8405,7 +8405,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -8570,7 +8570,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -8834,7 +8834,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -9234,7 +9234,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -9498,7 +9498,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -9531,7 +9531,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -9894,7 +9894,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -9960,7 +9960,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -10092,7 +10092,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -10356,7 +10356,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -11379,7 +11379,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -11412,7 +11412,7 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
@@ -11445,7 +11445,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
@@ -11709,7 +11709,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
@@ -11775,7 +11775,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
@@ -12406,7 +12406,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
@@ -12670,7 +12670,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
@@ -12905,7 +12905,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
@@ -12938,7 +12938,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D375" t="inlineStr">
@@ -13235,7 +13235,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
@@ -13334,7 +13334,7 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D381" t="inlineStr">
@@ -13499,7 +13499,7 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
@@ -13664,7 +13664,7 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
@@ -13730,7 +13730,7 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
@@ -13763,7 +13763,7 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
@@ -13994,7 +13994,7 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D401" t="inlineStr">
@@ -14027,7 +14027,7 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D402" t="inlineStr">
@@ -14192,7 +14192,7 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
@@ -14291,7 +14291,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
@@ -14592,7 +14592,7 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
@@ -15483,7 +15483,7 @@
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D446" t="inlineStr">
@@ -16015,7 +16015,7 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -16279,7 +16279,7 @@
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
@@ -16448,7 +16448,7 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
@@ -16580,7 +16580,7 @@
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
@@ -16613,7 +16613,7 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -16778,7 +16778,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -17042,7 +17042,7 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -17339,7 +17339,7 @@
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -17537,7 +17537,7 @@
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
@@ -17867,7 +17867,7 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
@@ -18201,7 +18201,7 @@
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
@@ -18432,7 +18432,7 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
@@ -18498,7 +18498,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
@@ -18564,7 +18564,7 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
@@ -18601,7 +18601,7 @@
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
@@ -18700,7 +18700,7 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D543" t="inlineStr">
@@ -18799,7 +18799,7 @@
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D546" t="inlineStr">
@@ -18832,7 +18832,7 @@
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D547" t="inlineStr">
@@ -19100,7 +19100,7 @@
       </c>
       <c r="C555" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D555" t="inlineStr">
@@ -19133,7 +19133,7 @@
       </c>
       <c r="C556" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D556" t="inlineStr">
@@ -19768,7 +19768,7 @@
       </c>
       <c r="C575" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D575" t="inlineStr">
@@ -19801,7 +19801,7 @@
       </c>
       <c r="C576" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D576" t="inlineStr">
@@ -20304,7 +20304,7 @@
       </c>
       <c r="C591" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D591" t="inlineStr">
@@ -20502,7 +20502,7 @@
       </c>
       <c r="C597" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D597" t="inlineStr">
@@ -20667,7 +20667,7 @@
       </c>
       <c r="C602" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D602" t="inlineStr">
@@ -20799,7 +20799,7 @@
       </c>
       <c r="C606" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D606" t="inlineStr">
@@ -20832,7 +20832,7 @@
       </c>
       <c r="C607" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D607" t="inlineStr">
@@ -20931,7 +20931,7 @@
       </c>
       <c r="C610" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D610" t="inlineStr">
@@ -20964,7 +20964,7 @@
       </c>
       <c r="C611" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D611" t="inlineStr">
@@ -20997,7 +20997,7 @@
       </c>
       <c r="C612" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D612" t="inlineStr">
@@ -21331,7 +21331,7 @@
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D622" t="inlineStr">
@@ -21463,7 +21463,7 @@
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
@@ -21801,7 +21801,7 @@
       </c>
       <c r="C636" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D636" t="inlineStr">
@@ -21999,7 +21999,7 @@
       </c>
       <c r="C642" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D642" t="inlineStr">
@@ -22032,7 +22032,7 @@
       </c>
       <c r="C643" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D643" t="inlineStr">
@@ -22098,7 +22098,7 @@
       </c>
       <c r="C645" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D645" t="inlineStr">
@@ -22329,7 +22329,7 @@
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D652" t="inlineStr">
@@ -22428,7 +22428,7 @@
       </c>
       <c r="C655" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D655" t="inlineStr">
@@ -22762,7 +22762,7 @@
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D665" t="inlineStr">
@@ -23191,7 +23191,7 @@
       </c>
       <c r="C678" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D678" t="inlineStr">
@@ -23727,7 +23727,7 @@
       </c>
       <c r="C694" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D694" t="inlineStr">
@@ -23793,7 +23793,7 @@
       </c>
       <c r="C696" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D696" t="inlineStr">
@@ -24123,7 +24123,7 @@
       </c>
       <c r="C706" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D706" t="inlineStr">
@@ -24189,7 +24189,7 @@
       </c>
       <c r="C708" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D708" t="inlineStr">
@@ -24354,7 +24354,7 @@
       </c>
       <c r="C713" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D713" t="inlineStr">
@@ -24420,7 +24420,7 @@
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
@@ -24618,7 +24618,7 @@
       </c>
       <c r="C721" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D721" t="inlineStr">
@@ -24783,7 +24783,7 @@
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
@@ -24820,7 +24820,7 @@
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
@@ -25117,7 +25117,7 @@
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D736" t="inlineStr">
@@ -25315,7 +25315,7 @@
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D742" t="inlineStr">
@@ -25579,7 +25579,7 @@
       </c>
       <c r="C750" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D750" t="inlineStr">
@@ -25645,7 +25645,7 @@
       </c>
       <c r="C752" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D752" t="inlineStr">
@@ -25711,7 +25711,7 @@
       </c>
       <c r="C754" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D754" t="inlineStr">
@@ -25744,7 +25744,7 @@
       </c>
       <c r="C755" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D755" t="inlineStr">
@@ -25810,7 +25810,7 @@
       </c>
       <c r="C757" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D757" t="inlineStr">
@@ -25843,7 +25843,7 @@
       </c>
       <c r="C758" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D758" t="inlineStr">
@@ -25909,7 +25909,7 @@
       </c>
       <c r="C760" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D760" t="inlineStr">
@@ -26074,7 +26074,7 @@
       </c>
       <c r="C765" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D765" t="inlineStr">
@@ -26144,7 +26144,7 @@
       </c>
       <c r="C767" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D767" t="inlineStr">
@@ -26639,7 +26639,7 @@
       </c>
       <c r="C782" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D782" t="inlineStr">
@@ -26672,7 +26672,7 @@
       </c>
       <c r="C783" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D783" t="inlineStr">
@@ -26738,7 +26738,7 @@
       </c>
       <c r="C785" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D785" t="inlineStr">
@@ -27237,7 +27237,7 @@
       </c>
       <c r="C800" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D800" t="inlineStr">
@@ -27336,7 +27336,7 @@
       </c>
       <c r="C803" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D803" t="inlineStr">
@@ -27600,7 +27600,7 @@
       </c>
       <c r="C811" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D811" t="inlineStr">
@@ -27765,7 +27765,7 @@
       </c>
       <c r="C816" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D816" t="inlineStr">
@@ -28194,7 +28194,7 @@
       </c>
       <c r="C829" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D829" t="inlineStr">
@@ -28392,7 +28392,7 @@
       </c>
       <c r="C835" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D835" t="inlineStr">
@@ -28722,7 +28722,7 @@
       </c>
       <c r="C845" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D845" t="inlineStr">
@@ -28887,7 +28887,7 @@
       </c>
       <c r="C850" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D850" t="inlineStr">
@@ -28986,7 +28986,7 @@
       </c>
       <c r="C853" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D853" t="inlineStr">
@@ -29188,7 +29188,7 @@
       </c>
       <c r="C859" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D859" t="inlineStr">
@@ -29423,7 +29423,7 @@
       </c>
       <c r="C866" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D866" t="inlineStr">
@@ -29460,7 +29460,7 @@
       </c>
       <c r="C867" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D867" t="inlineStr">
@@ -29530,7 +29530,7 @@
       </c>
       <c r="C869" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D869" t="inlineStr">
@@ -29992,7 +29992,7 @@
       </c>
       <c r="C883" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D883" t="inlineStr">
@@ -30322,7 +30322,7 @@
       </c>
       <c r="C893" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D893" t="inlineStr">
@@ -30454,7 +30454,7 @@
       </c>
       <c r="C897" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D897" t="inlineStr">
@@ -30553,7 +30553,7 @@
       </c>
       <c r="C900" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D900" t="inlineStr">
@@ -30652,7 +30652,7 @@
       </c>
       <c r="C903" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D903" t="inlineStr">
@@ -30817,7 +30817,7 @@
       </c>
       <c r="C908" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D908" t="inlineStr">
@@ -31147,7 +31147,7 @@
       </c>
       <c r="C918" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D918" t="inlineStr">
@@ -31213,7 +31213,7 @@
       </c>
       <c r="C920" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D920" t="inlineStr">
@@ -31246,7 +31246,7 @@
       </c>
       <c r="C921" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D921" t="inlineStr">
@@ -31312,7 +31312,7 @@
       </c>
       <c r="C923" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D923" t="inlineStr">
@@ -31444,7 +31444,7 @@
       </c>
       <c r="C927" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D927" t="inlineStr">
@@ -31576,7 +31576,7 @@
       </c>
       <c r="C931" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D931" t="inlineStr">
@@ -31609,7 +31609,7 @@
       </c>
       <c r="C932" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D932" t="inlineStr">
@@ -32038,7 +32038,7 @@
       </c>
       <c r="C945" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D945" t="inlineStr">
@@ -32203,7 +32203,7 @@
       </c>
       <c r="C950" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D950" t="inlineStr">
@@ -32269,7 +32269,7 @@
       </c>
       <c r="C952" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D952" t="inlineStr">
@@ -32335,7 +32335,7 @@
       </c>
       <c r="C954" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D954" t="inlineStr">
@@ -32434,7 +32434,7 @@
       </c>
       <c r="C957" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D957" t="inlineStr">
@@ -32566,7 +32566,7 @@
       </c>
       <c r="C961" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D961" t="inlineStr">
@@ -32863,7 +32863,7 @@
       </c>
       <c r="C970" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D970" t="inlineStr">
@@ -32929,7 +32929,7 @@
       </c>
       <c r="C972" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D972" t="inlineStr">
@@ -32962,7 +32962,7 @@
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D973" t="inlineStr">
@@ -33127,7 +33127,7 @@
       </c>
       <c r="C978" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D978" t="inlineStr">
@@ -33160,7 +33160,7 @@
       </c>
       <c r="C979" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D979" t="inlineStr">
@@ -33292,7 +33292,7 @@
       </c>
       <c r="C983" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D983" t="inlineStr">
@@ -33358,7 +33358,7 @@
       </c>
       <c r="C985" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D985" t="inlineStr">
@@ -33457,7 +33457,7 @@
       </c>
       <c r="C988" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D988" t="inlineStr">
@@ -33688,7 +33688,7 @@
       </c>
       <c r="C995" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D995" t="inlineStr">
@@ -33853,7 +33853,7 @@
       </c>
       <c r="C1000" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1000" t="inlineStr">
@@ -33886,7 +33886,7 @@
       </c>
       <c r="C1001" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1001" t="inlineStr">
@@ -34018,7 +34018,7 @@
       </c>
       <c r="C1005" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1005" t="inlineStr">
@@ -34084,7 +34084,7 @@
       </c>
       <c r="C1007" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1007" t="inlineStr">
@@ -34121,7 +34121,7 @@
       </c>
       <c r="C1008" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1008" t="inlineStr">
@@ -34319,7 +34319,7 @@
       </c>
       <c r="C1014" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1014" t="inlineStr">
@@ -34352,7 +34352,7 @@
       </c>
       <c r="C1015" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1015" t="inlineStr">
@@ -34616,7 +34616,7 @@
       </c>
       <c r="C1023" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1023" t="inlineStr">
@@ -34649,7 +34649,7 @@
       </c>
       <c r="C1024" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1024" t="inlineStr">
@@ -34979,7 +34979,7 @@
       </c>
       <c r="C1034" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1034" t="inlineStr">
@@ -35573,7 +35573,7 @@
       </c>
       <c r="C1052" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1052" t="inlineStr">
@@ -35837,7 +35837,7 @@
       </c>
       <c r="C1060" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1060" t="inlineStr">
@@ -35936,7 +35936,7 @@
       </c>
       <c r="C1063" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1063" t="inlineStr">
@@ -36505,7 +36505,7 @@
       </c>
       <c r="C1080" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1080" t="inlineStr">
@@ -36571,7 +36571,7 @@
       </c>
       <c r="C1082" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1082" t="inlineStr">
@@ -36637,7 +36637,7 @@
       </c>
       <c r="C1084" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1084" t="inlineStr">
@@ -36773,7 +36773,7 @@
       </c>
       <c r="C1088" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1088" t="inlineStr">
@@ -36872,7 +36872,7 @@
       </c>
       <c r="C1091" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1091" t="inlineStr">
@@ -36905,7 +36905,7 @@
       </c>
       <c r="C1092" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1092" t="inlineStr">
@@ -36938,7 +36938,7 @@
       </c>
       <c r="C1093" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1093" t="inlineStr">
@@ -37070,7 +37070,7 @@
       </c>
       <c r="C1097" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1097" t="inlineStr">
@@ -37404,7 +37404,7 @@
       </c>
       <c r="C1107" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1107" t="inlineStr">
@@ -37503,7 +37503,7 @@
       </c>
       <c r="C1110" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1110" t="inlineStr">
@@ -37701,7 +37701,7 @@
       </c>
       <c r="C1116" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1116" t="inlineStr">
@@ -37800,7 +37800,7 @@
       </c>
       <c r="C1119" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1119" t="inlineStr">
@@ -37833,7 +37833,7 @@
       </c>
       <c r="C1120" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1120" t="inlineStr">
@@ -38101,7 +38101,7 @@
       </c>
       <c r="C1128" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1128" t="inlineStr">
@@ -38233,7 +38233,7 @@
       </c>
       <c r="C1132" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1132" t="inlineStr">
@@ -38299,7 +38299,7 @@
       </c>
       <c r="C1134" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1134" t="inlineStr">
@@ -38468,7 +38468,7 @@
       </c>
       <c r="C1139" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1139" t="inlineStr">
@@ -39128,7 +39128,7 @@
       </c>
       <c r="C1159" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1159" t="inlineStr">
@@ -39194,7 +39194,7 @@
       </c>
       <c r="C1161" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1161" t="inlineStr">
@@ -39227,7 +39227,7 @@
       </c>
       <c r="C1162" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1162" t="inlineStr">
@@ -39326,7 +39326,7 @@
       </c>
       <c r="C1165" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1165" t="inlineStr">
@@ -39458,7 +39458,7 @@
       </c>
       <c r="C1169" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1169" t="inlineStr">
@@ -39524,7 +39524,7 @@
       </c>
       <c r="C1171" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1171" t="inlineStr">
@@ -40254,7 +40254,7 @@
       </c>
       <c r="C1193" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1193" t="inlineStr">
@@ -40390,7 +40390,7 @@
       </c>
       <c r="C1197" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1197" t="inlineStr">
@@ -40786,7 +40786,7 @@
       </c>
       <c r="C1209" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1209" t="inlineStr">
@@ -41050,7 +41050,7 @@
       </c>
       <c r="C1217" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1217" t="inlineStr">
@@ -41083,7 +41083,7 @@
       </c>
       <c r="C1218" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1218" t="inlineStr">
@@ -41149,7 +41149,7 @@
       </c>
       <c r="C1220" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1220" t="inlineStr">
@@ -41248,7 +41248,7 @@
       </c>
       <c r="C1223" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1223" t="inlineStr">
@@ -41842,7 +41842,7 @@
       </c>
       <c r="C1241" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1241" t="inlineStr">
@@ -42011,7 +42011,7 @@
       </c>
       <c r="C1246" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1246" t="inlineStr">
@@ -42044,7 +42044,7 @@
       </c>
       <c r="C1247" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1247" t="inlineStr">
@@ -42308,7 +42308,7 @@
       </c>
       <c r="C1255" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1255" t="inlineStr">
@@ -42341,7 +42341,7 @@
       </c>
       <c r="C1256" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1256" t="inlineStr">
@@ -42539,7 +42539,7 @@
       </c>
       <c r="C1262" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1262" t="inlineStr">
@@ -42638,7 +42638,7 @@
       </c>
       <c r="C1265" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1265" t="inlineStr">
@@ -42836,7 +42836,7 @@
       </c>
       <c r="C1271" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1271" t="inlineStr">
@@ -42968,7 +42968,7 @@
       </c>
       <c r="C1275" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1275" t="inlineStr">
@@ -43100,7 +43100,7 @@
       </c>
       <c r="C1279" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1279" t="inlineStr">
@@ -43170,7 +43170,7 @@
       </c>
       <c r="C1281" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1281" t="inlineStr">
@@ -43236,7 +43236,7 @@
       </c>
       <c r="C1283" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1283" t="inlineStr">
@@ -43368,7 +43368,7 @@
       </c>
       <c r="C1287" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1287" t="inlineStr">
@@ -43500,7 +43500,7 @@
       </c>
       <c r="C1291" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1291" t="inlineStr">
@@ -43999,7 +43999,7 @@
       </c>
       <c r="C1306" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1306" t="inlineStr">
@@ -44131,7 +44131,7 @@
       </c>
       <c r="C1310" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1310" t="inlineStr">
@@ -44197,7 +44197,7 @@
       </c>
       <c r="C1312" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1312" t="inlineStr">
@@ -44296,7 +44296,7 @@
       </c>
       <c r="C1315" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1315" t="inlineStr">
@@ -44564,7 +44564,7 @@
       </c>
       <c r="C1323" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1323" t="inlineStr">
@@ -44927,7 +44927,7 @@
       </c>
       <c r="C1334" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1334" t="inlineStr">
@@ -45191,7 +45191,7 @@
       </c>
       <c r="C1342" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1342" t="inlineStr">
@@ -45228,7 +45228,7 @@
       </c>
       <c r="C1343" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1343" t="inlineStr">
@@ -45261,7 +45261,7 @@
       </c>
       <c r="C1344" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1344" t="inlineStr">
@@ -45393,7 +45393,7 @@
       </c>
       <c r="C1348" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1348" t="inlineStr">
@@ -45690,7 +45690,7 @@
       </c>
       <c r="C1357" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1357" t="inlineStr">
@@ -45793,7 +45793,7 @@
       </c>
       <c r="C1360" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1360" t="inlineStr">
@@ -45826,7 +45826,7 @@
       </c>
       <c r="C1361" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1361" t="inlineStr">
@@ -45995,7 +45995,7 @@
       </c>
       <c r="C1366" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1366" t="inlineStr">
@@ -46094,7 +46094,7 @@
       </c>
       <c r="C1369" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1369" t="inlineStr">
@@ -46329,7 +46329,7 @@
       </c>
       <c r="C1376" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1376" t="inlineStr">
@@ -46494,7 +46494,7 @@
       </c>
       <c r="C1381" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1381" t="inlineStr">
@@ -46560,7 +46560,7 @@
       </c>
       <c r="C1383" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1383" t="inlineStr">
@@ -47154,7 +47154,7 @@
       </c>
       <c r="C1401" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1401" t="inlineStr">
@@ -47220,7 +47220,7 @@
       </c>
       <c r="C1403" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1403" t="inlineStr">
@@ -47319,7 +47319,7 @@
       </c>
       <c r="C1406" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1406" t="inlineStr">
@@ -47649,7 +47649,7 @@
       </c>
       <c r="C1416" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1416" t="inlineStr">
@@ -47715,7 +47715,7 @@
       </c>
       <c r="C1418" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1418" t="inlineStr">
@@ -47781,7 +47781,7 @@
       </c>
       <c r="C1420" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1420" t="inlineStr">
@@ -48144,7 +48144,7 @@
       </c>
       <c r="C1431" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1431" t="inlineStr">
@@ -48210,7 +48210,7 @@
       </c>
       <c r="C1433" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1433" t="inlineStr">
@@ -48507,7 +48507,7 @@
       </c>
       <c r="C1442" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1442" t="inlineStr">
@@ -48540,7 +48540,7 @@
       </c>
       <c r="C1443" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1443" t="inlineStr">
@@ -48705,7 +48705,7 @@
       </c>
       <c r="C1448" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1448" t="inlineStr">
@@ -48837,7 +48837,7 @@
       </c>
       <c r="C1452" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1452" t="inlineStr">
@@ -48969,7 +48969,7 @@
       </c>
       <c r="C1456" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1456" t="inlineStr">
@@ -49233,7 +49233,7 @@
       </c>
       <c r="C1464" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1464" t="inlineStr">
@@ -49266,7 +49266,7 @@
       </c>
       <c r="C1465" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1465" t="inlineStr">
@@ -49365,7 +49365,7 @@
       </c>
       <c r="C1468" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1468" t="inlineStr">
@@ -49530,7 +49530,7 @@
       </c>
       <c r="C1473" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1473" t="inlineStr">
@@ -49563,7 +49563,7 @@
       </c>
       <c r="C1474" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1474" t="inlineStr">
@@ -49596,7 +49596,7 @@
       </c>
       <c r="C1475" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1475" t="inlineStr">
@@ -49761,7 +49761,7 @@
       </c>
       <c r="C1480" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1480" t="inlineStr">
@@ -49963,7 +49963,7 @@
       </c>
       <c r="C1486" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1486" t="inlineStr">
@@ -50095,7 +50095,7 @@
       </c>
       <c r="C1490" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1490" t="inlineStr">
@@ -50227,7 +50227,7 @@
       </c>
       <c r="C1494" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1494" t="inlineStr">
@@ -50326,7 +50326,7 @@
       </c>
       <c r="C1497" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1497" t="inlineStr">
@@ -50594,7 +50594,7 @@
       </c>
       <c r="C1505" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1505" t="inlineStr">
@@ -50924,7 +50924,7 @@
       </c>
       <c r="C1515" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1515" t="inlineStr">
@@ -50957,7 +50957,7 @@
       </c>
       <c r="C1516" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1516" t="inlineStr">
@@ -50990,7 +50990,7 @@
       </c>
       <c r="C1517" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1517" t="inlineStr">
@@ -51254,7 +51254,7 @@
       </c>
       <c r="C1525" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1525" t="inlineStr">
@@ -51353,7 +51353,7 @@
       </c>
       <c r="C1528" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1528" t="inlineStr">
@@ -51452,7 +51452,7 @@
       </c>
       <c r="C1531" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1531" t="inlineStr">
@@ -51551,7 +51551,7 @@
       </c>
       <c r="C1534" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1534" t="inlineStr">
@@ -51683,7 +51683,7 @@
       </c>
       <c r="C1538" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1538" t="inlineStr">
@@ -51815,7 +51815,7 @@
       </c>
       <c r="C1542" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1542" t="inlineStr">
@@ -51984,7 +51984,7 @@
       </c>
       <c r="C1547" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1547" t="inlineStr">
@@ -52149,7 +52149,7 @@
       </c>
       <c r="C1552" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1552" t="inlineStr">
@@ -52413,7 +52413,7 @@
       </c>
       <c r="C1560" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1560" t="inlineStr">
@@ -52446,7 +52446,7 @@
       </c>
       <c r="C1561" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1561" t="inlineStr">
@@ -52479,7 +52479,7 @@
       </c>
       <c r="C1562" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1562" t="inlineStr">
@@ -52776,7 +52776,7 @@
       </c>
       <c r="C1571" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1571" t="inlineStr">
@@ -52809,7 +52809,7 @@
       </c>
       <c r="C1572" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1572" t="inlineStr">
@@ -52875,7 +52875,7 @@
       </c>
       <c r="C1574" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1574" t="inlineStr">
@@ -53040,7 +53040,7 @@
       </c>
       <c r="C1579" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1579" t="inlineStr">
@@ -53213,7 +53213,7 @@
       </c>
       <c r="C1584" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1584" t="inlineStr">
@@ -53283,7 +53283,7 @@
       </c>
       <c r="C1586" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1586" t="inlineStr">
@@ -53646,7 +53646,7 @@
       </c>
       <c r="C1597" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1597" t="inlineStr">
@@ -53679,7 +53679,7 @@
       </c>
       <c r="C1598" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1598" t="inlineStr">
@@ -53811,7 +53811,7 @@
       </c>
       <c r="C1602" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1602" t="inlineStr">
@@ -53976,7 +53976,7 @@
       </c>
       <c r="C1607" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1607" t="inlineStr">
@@ -54075,7 +54075,7 @@
       </c>
       <c r="C1610" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1610" t="inlineStr">
@@ -54405,7 +54405,7 @@
       </c>
       <c r="C1620" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1620" t="inlineStr">
@@ -54537,7 +54537,7 @@
       </c>
       <c r="C1624" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1624" t="inlineStr">
@@ -54834,7 +54834,7 @@
       </c>
       <c r="C1633" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1633" t="inlineStr">
@@ -55036,7 +55036,7 @@
       </c>
       <c r="C1639" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1639" t="inlineStr">
@@ -55135,7 +55135,7 @@
       </c>
       <c r="C1642" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1642" t="inlineStr">
@@ -55366,7 +55366,7 @@
       </c>
       <c r="C1649" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1649" t="inlineStr">
@@ -55795,7 +55795,7 @@
       </c>
       <c r="C1662" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1662" t="inlineStr">
@@ -55828,7 +55828,7 @@
       </c>
       <c r="C1663" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1663" t="inlineStr">
@@ -55861,7 +55861,7 @@
       </c>
       <c r="C1664" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1664" t="inlineStr">
@@ -56529,7 +56529,7 @@
       </c>
       <c r="C1684" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1684" t="inlineStr">
@@ -56595,7 +56595,7 @@
       </c>
       <c r="C1686" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1686" t="inlineStr">
@@ -56925,7 +56925,7 @@
       </c>
       <c r="C1696" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1696" t="inlineStr">
@@ -57057,7 +57057,7 @@
       </c>
       <c r="C1700" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1700" t="inlineStr">
@@ -57123,7 +57123,7 @@
       </c>
       <c r="C1702" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1702" t="inlineStr">
@@ -57255,7 +57255,7 @@
       </c>
       <c r="C1706" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1706" t="inlineStr">
@@ -57288,7 +57288,7 @@
       </c>
       <c r="C1707" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1707" t="inlineStr">
@@ -57453,7 +57453,7 @@
       </c>
       <c r="C1712" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1712" t="inlineStr">
@@ -57552,7 +57552,7 @@
       </c>
       <c r="C1715" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1715" t="inlineStr">
@@ -57651,7 +57651,7 @@
       </c>
       <c r="C1718" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1718" t="inlineStr">
@@ -57750,7 +57750,7 @@
       </c>
       <c r="C1721" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1721" t="inlineStr">
@@ -57849,7 +57849,7 @@
       </c>
       <c r="C1724" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1724" t="inlineStr">
@@ -57915,7 +57915,7 @@
       </c>
       <c r="C1726" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1726" t="inlineStr">
@@ -58150,7 +58150,7 @@
       </c>
       <c r="C1733" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1733" t="inlineStr">
@@ -58381,7 +58381,7 @@
       </c>
       <c r="C1740" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1740" t="inlineStr">
@@ -58546,7 +58546,7 @@
       </c>
       <c r="C1745" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1745" t="inlineStr">
@@ -58645,7 +58645,7 @@
       </c>
       <c r="C1748" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1748" t="inlineStr">
@@ -58678,7 +58678,7 @@
       </c>
       <c r="C1749" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1749" t="inlineStr">
@@ -58810,7 +58810,7 @@
       </c>
       <c r="C1753" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1753" t="inlineStr">
@@ -58942,7 +58942,7 @@
       </c>
       <c r="C1757" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1757" t="inlineStr">
@@ -59243,7 +59243,7 @@
       </c>
       <c r="C1766" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1766" t="inlineStr">
@@ -59540,7 +59540,7 @@
       </c>
       <c r="C1775" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1775" t="inlineStr">
@@ -59738,7 +59738,7 @@
       </c>
       <c r="C1781" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1781" t="inlineStr">
@@ -59969,7 +59969,7 @@
       </c>
       <c r="C1788" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1788" t="inlineStr">
@@ -60266,7 +60266,7 @@
       </c>
       <c r="C1797" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1797" t="inlineStr">
@@ -60299,7 +60299,7 @@
       </c>
       <c r="C1798" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1798" t="inlineStr">
@@ -60497,7 +60497,7 @@
       </c>
       <c r="C1804" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1804" t="inlineStr">
@@ -60695,7 +60695,7 @@
       </c>
       <c r="C1810" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1810" t="inlineStr">
@@ -61025,7 +61025,7 @@
       </c>
       <c r="C1820" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1820" t="inlineStr">
@@ -61355,7 +61355,7 @@
       </c>
       <c r="C1830" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1830" t="inlineStr">
@@ -61421,7 +61421,7 @@
       </c>
       <c r="C1832" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1832" t="inlineStr">
@@ -61590,7 +61590,7 @@
       </c>
       <c r="C1837" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1837" t="inlineStr">
@@ -61722,7 +61722,7 @@
       </c>
       <c r="C1841" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1841" t="inlineStr">
@@ -61825,7 +61825,7 @@
       </c>
       <c r="C1844" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1844" t="inlineStr">
@@ -62126,7 +62126,7 @@
       </c>
       <c r="C1853" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1853" t="inlineStr">
@@ -62159,7 +62159,7 @@
       </c>
       <c r="C1854" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1854" t="inlineStr">
@@ -62192,7 +62192,7 @@
       </c>
       <c r="C1855" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1855" t="inlineStr">
@@ -62328,7 +62328,7 @@
       </c>
       <c r="C1859" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1859" t="inlineStr">
@@ -62460,7 +62460,7 @@
       </c>
       <c r="C1863" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1863" t="inlineStr">
@@ -62493,7 +62493,7 @@
       </c>
       <c r="C1864" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1864" t="inlineStr">
@@ -62592,7 +62592,7 @@
       </c>
       <c r="C1867" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1867" t="inlineStr">
@@ -62988,7 +62988,7 @@
       </c>
       <c r="C1879" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1879" t="inlineStr">
@@ -63021,7 +63021,7 @@
       </c>
       <c r="C1880" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1880" t="inlineStr">
@@ -63417,7 +63417,7 @@
       </c>
       <c r="C1892" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1892" t="inlineStr">
@@ -63450,7 +63450,7 @@
       </c>
       <c r="C1893" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1893" t="inlineStr">
@@ -63714,7 +63714,7 @@
       </c>
       <c r="C1901" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1901" t="inlineStr">
@@ -64044,7 +64044,7 @@
       </c>
       <c r="C1911" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1911" t="inlineStr">
@@ -64209,7 +64209,7 @@
       </c>
       <c r="C1916" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1916" t="inlineStr">
@@ -64308,7 +64308,7 @@
       </c>
       <c r="C1919" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1919" t="inlineStr">
@@ -64741,7 +64741,7 @@
       </c>
       <c r="C1932" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1932" t="inlineStr">
@@ -64873,7 +64873,7 @@
       </c>
       <c r="C1936" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1936" t="inlineStr">
@@ -65038,7 +65038,7 @@
       </c>
       <c r="C1941" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1941" t="inlineStr">
@@ -65504,7 +65504,7 @@
       </c>
       <c r="C1955" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1955" t="inlineStr">
@@ -65541,7 +65541,7 @@
       </c>
       <c r="C1956" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1956" t="inlineStr">
@@ -65607,7 +65607,7 @@
       </c>
       <c r="C1958" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1958" t="inlineStr">
@@ -65673,7 +65673,7 @@
       </c>
       <c r="C1960" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1960" t="inlineStr">
@@ -65706,7 +65706,7 @@
       </c>
       <c r="C1961" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1961" t="inlineStr">
@@ -65871,7 +65871,7 @@
       </c>
       <c r="C1966" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1966" t="inlineStr">
@@ -65904,7 +65904,7 @@
       </c>
       <c r="C1967" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1967" t="inlineStr">
@@ -66036,7 +66036,7 @@
       </c>
       <c r="C1971" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1971" t="inlineStr">
@@ -66201,7 +66201,7 @@
       </c>
       <c r="C1976" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1976" t="inlineStr">
@@ -66601,7 +66601,7 @@
       </c>
       <c r="C1988" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1988" t="inlineStr">
@@ -66807,7 +66807,7 @@
       </c>
       <c r="C1994" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D1994" t="inlineStr">
@@ -66840,7 +66840,7 @@
       </c>
       <c r="C1995" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1995" t="inlineStr">
@@ -66873,7 +66873,7 @@
       </c>
       <c r="C1996" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D1996" t="inlineStr">
@@ -67401,7 +67401,7 @@
       </c>
       <c r="C2012" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2012" t="inlineStr">
@@ -67434,7 +67434,7 @@
       </c>
       <c r="C2013" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2013" t="inlineStr">
@@ -67467,7 +67467,7 @@
       </c>
       <c r="C2014" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2014" t="inlineStr">
@@ -67570,7 +67570,7 @@
       </c>
       <c r="C2017" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2017" t="inlineStr">
@@ -67636,7 +67636,7 @@
       </c>
       <c r="C2019" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2019" t="inlineStr">
@@ -67702,7 +67702,7 @@
       </c>
       <c r="C2021" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2021" t="inlineStr">
@@ -67904,7 +67904,7 @@
       </c>
       <c r="C2027" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2027" t="inlineStr">
@@ -68069,7 +68069,7 @@
       </c>
       <c r="C2032" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2032" t="inlineStr">
@@ -68102,7 +68102,7 @@
       </c>
       <c r="C2033" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2033" t="inlineStr">
@@ -68139,7 +68139,7 @@
       </c>
       <c r="C2034" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2034" t="inlineStr">
@@ -68209,7 +68209,7 @@
       </c>
       <c r="C2036" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2036" t="inlineStr">
@@ -68275,7 +68275,7 @@
       </c>
       <c r="C2038" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2038" t="inlineStr">
@@ -68671,7 +68671,7 @@
       </c>
       <c r="C2050" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2050" t="inlineStr">
@@ -68704,7 +68704,7 @@
       </c>
       <c r="C2051" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2051" t="inlineStr">
@@ -68935,7 +68935,7 @@
       </c>
       <c r="C2058" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2058" t="inlineStr">
@@ -69430,7 +69430,7 @@
       </c>
       <c r="C2073" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2073" t="inlineStr">
@@ -69665,7 +69665,7 @@
       </c>
       <c r="C2080" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2080" t="inlineStr">
@@ -69698,7 +69698,7 @@
       </c>
       <c r="C2081" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2081" t="inlineStr">
@@ -70193,7 +70193,7 @@
       </c>
       <c r="C2096" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2096" t="inlineStr">
@@ -70259,7 +70259,7 @@
       </c>
       <c r="C2098" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2098" t="inlineStr">
@@ -70721,7 +70721,7 @@
       </c>
       <c r="C2112" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2112" t="inlineStr">
@@ -70923,7 +70923,7 @@
       </c>
       <c r="C2118" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2118" t="inlineStr">
@@ -70989,7 +70989,7 @@
       </c>
       <c r="C2120" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2120" t="inlineStr">
@@ -71022,7 +71022,7 @@
       </c>
       <c r="C2121" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2121" t="inlineStr">
@@ -71253,7 +71253,7 @@
       </c>
       <c r="C2128" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2128" t="inlineStr">
@@ -71319,7 +71319,7 @@
       </c>
       <c r="C2130" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2130" t="inlineStr">
@@ -71785,7 +71785,7 @@
       </c>
       <c r="C2144" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2144" t="inlineStr">
@@ -71884,7 +71884,7 @@
       </c>
       <c r="C2147" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2147" t="inlineStr">
@@ -72016,7 +72016,7 @@
       </c>
       <c r="C2151" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2151" t="inlineStr">
@@ -72148,7 +72148,7 @@
       </c>
       <c r="C2155" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2155" t="inlineStr">
@@ -72218,7 +72218,7 @@
       </c>
       <c r="C2157" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2157" t="inlineStr">
@@ -72354,7 +72354,7 @@
       </c>
       <c r="C2161" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2161" t="inlineStr">
@@ -72387,7 +72387,7 @@
       </c>
       <c r="C2162" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2162" t="inlineStr">
@@ -72486,7 +72486,7 @@
       </c>
       <c r="C2165" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2165" t="inlineStr">
@@ -72618,7 +72618,7 @@
       </c>
       <c r="C2169" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2169" t="inlineStr">
@@ -72717,7 +72717,7 @@
       </c>
       <c r="C2172" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2172" t="inlineStr">
@@ -72750,7 +72750,7 @@
       </c>
       <c r="C2173" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2173" t="inlineStr">
@@ -73113,7 +73113,7 @@
       </c>
       <c r="C2184" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2184" t="inlineStr">
@@ -73146,7 +73146,7 @@
       </c>
       <c r="C2185" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2185" t="inlineStr">
@@ -73245,7 +73245,7 @@
       </c>
       <c r="C2188" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2188" t="inlineStr">
@@ -73278,7 +73278,7 @@
       </c>
       <c r="C2189" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2189" t="inlineStr">
@@ -73542,7 +73542,7 @@
       </c>
       <c r="C2197" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2197" t="inlineStr">
@@ -73872,7 +73872,7 @@
       </c>
       <c r="C2207" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2207" t="inlineStr">
@@ -74037,7 +74037,7 @@
       </c>
       <c r="C2212" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2212" t="inlineStr">
@@ -74202,7 +74202,7 @@
       </c>
       <c r="C2217" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2217" t="inlineStr">
@@ -74301,7 +74301,7 @@
       </c>
       <c r="C2220" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2220" t="inlineStr">
@@ -74899,7 +74899,7 @@
       </c>
       <c r="C2238" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2238" t="inlineStr">
@@ -75031,7 +75031,7 @@
       </c>
       <c r="C2242" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2242" t="inlineStr">
@@ -75596,7 +75596,7 @@
       </c>
       <c r="C2259" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2259" t="inlineStr">
@@ -75695,7 +75695,7 @@
       </c>
       <c r="C2262" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2262" t="inlineStr">
@@ -75728,7 +75728,7 @@
       </c>
       <c r="C2263" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2263" t="inlineStr">
@@ -75963,7 +75963,7 @@
       </c>
       <c r="C2270" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2270" t="inlineStr">
@@ -76029,7 +76029,7 @@
       </c>
       <c r="C2272" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2272" t="inlineStr">
@@ -76095,7 +76095,7 @@
       </c>
       <c r="C2274" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2274" t="inlineStr">
@@ -76264,7 +76264,7 @@
       </c>
       <c r="C2279" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2279" t="inlineStr">
@@ -76363,7 +76363,7 @@
       </c>
       <c r="C2282" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2282" t="inlineStr">
@@ -76895,7 +76895,7 @@
       </c>
       <c r="C2298" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2298" t="inlineStr">
@@ -77225,7 +77225,7 @@
       </c>
       <c r="C2308" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2308" t="inlineStr">
@@ -77291,7 +77291,7 @@
       </c>
       <c r="C2310" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2310" t="inlineStr">
@@ -77357,7 +77357,7 @@
       </c>
       <c r="C2312" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2312" t="inlineStr">
@@ -77423,7 +77423,7 @@
       </c>
       <c r="C2314" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2314" t="inlineStr">
@@ -77761,7 +77761,7 @@
       </c>
       <c r="C2324" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2324" t="inlineStr">
@@ -77992,7 +77992,7 @@
       </c>
       <c r="C2331" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2331" t="inlineStr">
@@ -78553,7 +78553,7 @@
       </c>
       <c r="C2348" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2348" t="inlineStr">
@@ -78652,7 +78652,7 @@
       </c>
       <c r="C2351" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2351" t="inlineStr">
@@ -78689,7 +78689,7 @@
       </c>
       <c r="C2352" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2352" t="inlineStr">
@@ -78792,7 +78792,7 @@
       </c>
       <c r="C2355" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2355" t="inlineStr">
@@ -78825,7 +78825,7 @@
       </c>
       <c r="C2356" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2356" t="inlineStr">
@@ -79056,7 +79056,7 @@
       </c>
       <c r="C2363" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2363" t="inlineStr">
@@ -79122,7 +79122,7 @@
       </c>
       <c r="C2365" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2365" t="inlineStr">
@@ -79192,7 +79192,7 @@
       </c>
       <c r="C2367" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2367" t="inlineStr">
@@ -79225,7 +79225,7 @@
       </c>
       <c r="C2368" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2368" t="inlineStr">
@@ -79456,7 +79456,7 @@
       </c>
       <c r="C2375" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2375" t="inlineStr">
@@ -79489,7 +79489,7 @@
       </c>
       <c r="C2376" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2376" t="inlineStr">
@@ -79522,7 +79522,7 @@
       </c>
       <c r="C2377" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2377" t="inlineStr">
@@ -79786,7 +79786,7 @@
       </c>
       <c r="C2385" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2385" t="inlineStr">
@@ -79819,7 +79819,7 @@
       </c>
       <c r="C2386" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2386" t="inlineStr">
@@ -79852,7 +79852,7 @@
       </c>
       <c r="C2387" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2387" t="inlineStr">
@@ -79955,7 +79955,7 @@
       </c>
       <c r="C2390" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2390" t="inlineStr">
@@ -80219,7 +80219,7 @@
       </c>
       <c r="C2398" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2398" t="inlineStr">
@@ -80450,7 +80450,7 @@
       </c>
       <c r="C2405" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2405" t="inlineStr">
@@ -80615,7 +80615,7 @@
       </c>
       <c r="C2410" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2410" t="inlineStr">
@@ -80648,7 +80648,7 @@
       </c>
       <c r="C2411" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2411" t="inlineStr">
@@ -80681,7 +80681,7 @@
       </c>
       <c r="C2412" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2412" t="inlineStr">
@@ -81015,7 +81015,7 @@
       </c>
       <c r="C2422" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2422" t="inlineStr">
@@ -81048,7 +81048,7 @@
       </c>
       <c r="C2423" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2423" t="inlineStr">
@@ -81147,7 +81147,7 @@
       </c>
       <c r="C2426" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2426" t="inlineStr">
@@ -81312,7 +81312,7 @@
       </c>
       <c r="C2431" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2431" t="inlineStr">
@@ -81345,7 +81345,7 @@
       </c>
       <c r="C2432" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2432" t="inlineStr">
@@ -81514,7 +81514,7 @@
       </c>
       <c r="C2437" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2437" t="inlineStr">
@@ -81646,7 +81646,7 @@
       </c>
       <c r="C2441" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2441" t="inlineStr">
@@ -82141,7 +82141,7 @@
       </c>
       <c r="C2456" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2456" t="inlineStr">
@@ -82273,7 +82273,7 @@
       </c>
       <c r="C2460" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2460" t="inlineStr">
@@ -82306,7 +82306,7 @@
       </c>
       <c r="C2461" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2461" t="inlineStr">
@@ -82376,7 +82376,7 @@
       </c>
       <c r="C2463" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2463" t="inlineStr">
@@ -82442,7 +82442,7 @@
       </c>
       <c r="C2465" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2465" t="inlineStr">
@@ -82508,7 +82508,7 @@
       </c>
       <c r="C2467" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2467" t="inlineStr">
@@ -82541,7 +82541,7 @@
       </c>
       <c r="C2468" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2468" t="inlineStr">
@@ -82640,7 +82640,7 @@
       </c>
       <c r="C2471" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2471" t="inlineStr">
@@ -82673,7 +82673,7 @@
       </c>
       <c r="C2472" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2472" t="inlineStr">
@@ -82772,7 +82772,7 @@
       </c>
       <c r="C2475" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2475" t="inlineStr">
@@ -82805,7 +82805,7 @@
       </c>
       <c r="C2476" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2476" t="inlineStr">
@@ -82838,7 +82838,7 @@
       </c>
       <c r="C2477" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2477" t="inlineStr">
@@ -82871,7 +82871,7 @@
       </c>
       <c r="C2478" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2478" t="inlineStr">
@@ -83003,7 +83003,7 @@
       </c>
       <c r="C2482" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2482" t="inlineStr">
@@ -83135,7 +83135,7 @@
       </c>
       <c r="C2486" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2486" t="inlineStr">
@@ -83201,7 +83201,7 @@
       </c>
       <c r="C2488" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2488" t="inlineStr">
@@ -83366,7 +83366,7 @@
       </c>
       <c r="C2493" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2493" t="inlineStr">
@@ -83696,7 +83696,7 @@
       </c>
       <c r="C2503" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2503" t="inlineStr">
@@ -83762,7 +83762,7 @@
       </c>
       <c r="C2505" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2505" t="inlineStr">
@@ -83927,7 +83927,7 @@
       </c>
       <c r="C2510" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2510" t="inlineStr">
@@ -83960,7 +83960,7 @@
       </c>
       <c r="C2511" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2511" t="inlineStr">
@@ -83993,7 +83993,7 @@
       </c>
       <c r="C2512" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2512" t="inlineStr">
@@ -84026,7 +84026,7 @@
       </c>
       <c r="C2513" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2513" t="inlineStr">
@@ -84125,7 +84125,7 @@
       </c>
       <c r="C2516" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2516" t="inlineStr">
@@ -84158,7 +84158,7 @@
       </c>
       <c r="C2517" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2517" t="inlineStr">
@@ -84389,7 +84389,7 @@
       </c>
       <c r="C2524" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2524" t="inlineStr">
@@ -84422,7 +84422,7 @@
       </c>
       <c r="C2525" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2525" t="inlineStr">
@@ -84558,7 +84558,7 @@
       </c>
       <c r="C2529" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2529" t="inlineStr">
@@ -84591,7 +84591,7 @@
       </c>
       <c r="C2530" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2530" t="inlineStr">
@@ -85020,7 +85020,7 @@
       </c>
       <c r="C2543" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2543" t="inlineStr">
@@ -85317,7 +85317,7 @@
       </c>
       <c r="C2552" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2552" t="inlineStr">
@@ -85449,7 +85449,7 @@
       </c>
       <c r="C2556" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2556" t="inlineStr">
@@ -85585,7 +85585,7 @@
       </c>
       <c r="C2560" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2560" t="inlineStr">
@@ -85618,7 +85618,7 @@
       </c>
       <c r="C2561" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2561" t="inlineStr">
@@ -85725,7 +85725,7 @@
       </c>
       <c r="C2564" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2564" t="inlineStr">
@@ -85791,7 +85791,7 @@
       </c>
       <c r="C2566" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2566" t="inlineStr">
@@ -86092,7 +86092,7 @@
       </c>
       <c r="C2575" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2575" t="inlineStr">
@@ -86521,7 +86521,7 @@
       </c>
       <c r="C2588" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2588" t="inlineStr">
@@ -86752,7 +86752,7 @@
       </c>
       <c r="C2595" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2595" t="inlineStr">
@@ -86785,7 +86785,7 @@
       </c>
       <c r="C2596" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2596" t="inlineStr">
@@ -86851,7 +86851,7 @@
       </c>
       <c r="C2598" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2598" t="inlineStr">
@@ -86917,7 +86917,7 @@
       </c>
       <c r="C2600" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2600" t="inlineStr">
@@ -87181,7 +87181,7 @@
       </c>
       <c r="C2608" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2608" t="inlineStr">
@@ -87247,7 +87247,7 @@
       </c>
       <c r="C2610" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2610" t="inlineStr">
@@ -87280,7 +87280,7 @@
       </c>
       <c r="C2611" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D2611" t="inlineStr">
@@ -87445,7 +87445,7 @@
       </c>
       <c r="C2616" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2616" t="inlineStr">
@@ -87511,7 +87511,7 @@
       </c>
       <c r="C2618" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D2618" t="inlineStr">
@@ -87705,7 +87705,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -87718,14 +87718,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hr - Expense</t>
+          <t>HR - Expense</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>It</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -87738,7 +87738,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>It - Expense</t>
+          <t>IT - Expense</t>
         </is>
       </c>
     </row>

</xml_diff>